<commit_message>
feat(user-management): email verification, profile update, address book
Closes out the Authentication & User Management roadmap step (1.7 Product
Roadmap section 5) before moving to Product Catalog & Marketplace.

- Wire up MustVerifyEmail on User (was inert); login now blocks unverified
  accounts per the login user flow. Custom verify/resend endpoints since
  this is a public API-only backend, not session-gated like Laravel's
  stock EmailVerificationRequest.
- PATCH /account/profile (name/phone) and full address book CRUD
  (/account/addresses) with ownership checks and default-address logic.
- Fix a latent bug in the existing forgot-password flow: Password::
  sendResetLink() would 500 on first real send because the default
  ResetPassword notification needs a password.reset named route that
  doesn't exist here. Point it at the Next.js /reset-password page instead.
- Add PHPUnit feature tests (15 new, 17 total) covering both flows.
</commit_message>
<xml_diff>
--- a/Required Document/Roadmap_Website_Harmoni_Clothing.xlsx
+++ b/Required Document/Roadmap_Website_Harmoni_Clothing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Harmoni Clothing\Required Document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33ECAFFE-D5D0-4E40-85EF-C421D64826BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87A00537-192A-410D-B2F9-CCBCF56F412D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1064,15 +1064,6 @@
     <xf numFmtId="9" fontId="8" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1094,34 +1085,29 @@
     <xf numFmtId="0" fontId="14" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="43">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE5A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="9">
     <dxf>
       <font>
         <color rgb="FFB10202"/>
@@ -1184,266 +1170,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD4EDBC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE5A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD4EDBC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD4EDBC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2068,1482 +1794,1482 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="10" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="16">
+      <c r="B2" s="11">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="D2" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="16" t="s">
+      <c r="F2" s="11" t="s">
         <v>9</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H2" s="18"/>
+      <c r="H2" s="13"/>
     </row>
     <row r="3" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A3" s="21"/>
-      <c r="B3" s="16">
+      <c r="A3" s="17"/>
+      <c r="B3" s="11">
         <v>1.2</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="17" t="s">
+      <c r="E3" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="11" t="s">
         <v>15</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H3" s="18"/>
+      <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A4" s="21"/>
-      <c r="B4" s="16">
+      <c r="A4" s="17"/>
+      <c r="B4" s="11">
         <v>1.3</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="E4" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="11" t="s">
         <v>18</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H4" s="18"/>
+      <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A5" s="21"/>
-      <c r="B5" s="16">
+      <c r="A5" s="17"/>
+      <c r="B5" s="11">
         <v>1.4</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="11" t="s">
         <v>21</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="13"/>
     </row>
     <row r="6" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A6" s="21"/>
-      <c r="B6" s="16">
+      <c r="A6" s="17"/>
+      <c r="B6" s="11">
         <v>1.5</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="D6" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="F6" s="11" t="s">
         <v>24</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H6" s="18"/>
+      <c r="H6" s="13"/>
     </row>
     <row r="7" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A7" s="21"/>
-      <c r="B7" s="16">
+      <c r="A7" s="17"/>
+      <c r="B7" s="11">
         <v>1.6</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="F7" s="11" t="s">
         <v>27</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H7" s="18"/>
+      <c r="H7" s="13"/>
     </row>
     <row r="8" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A8" s="23"/>
-      <c r="B8" s="16">
+      <c r="A8" s="18"/>
+      <c r="B8" s="11">
         <v>1.7</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F8" s="11" t="s">
         <v>30</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H8" s="18"/>
+      <c r="H8" s="13"/>
     </row>
     <row r="9" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="11">
         <v>2.1</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="17" t="s">
+      <c r="E9" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="F9" s="11" t="s">
         <v>32</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H9" s="18"/>
+      <c r="H9" s="13"/>
     </row>
     <row r="10" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A10" s="21"/>
-      <c r="B10" s="16">
+      <c r="A10" s="17"/>
+      <c r="B10" s="11">
         <v>2.2000000000000002</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="16" t="s">
+      <c r="F10" s="11" t="s">
         <v>36</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H10" s="18"/>
+      <c r="H10" s="13"/>
     </row>
     <row r="11" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A11" s="21"/>
-      <c r="B11" s="16">
+      <c r="A11" s="17"/>
+      <c r="B11" s="11">
         <v>2.2999999999999998</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="F11" s="11" t="s">
         <v>39</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H11" s="18"/>
+      <c r="H11" s="13"/>
     </row>
     <row r="12" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A12" s="21"/>
-      <c r="B12" s="16">
+      <c r="A12" s="17"/>
+      <c r="B12" s="11">
         <v>2.4</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="16" t="s">
+      <c r="D12" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="E12" s="17" t="s">
+      <c r="E12" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F12" s="16" t="s">
+      <c r="F12" s="11" t="s">
         <v>42</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H12" s="18"/>
+      <c r="H12" s="13"/>
     </row>
     <row r="13" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A13" s="23"/>
-      <c r="B13" s="16">
+      <c r="A13" s="18"/>
+      <c r="B13" s="11">
         <v>2.5</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="E13" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F13" s="16" t="s">
+      <c r="F13" s="11" t="s">
         <v>43</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H13" s="18"/>
+      <c r="H13" s="13"/>
     </row>
     <row r="14" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="11">
         <v>3.1</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F14" s="16" t="s">
+      <c r="F14" s="11" t="s">
         <v>48</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H14" s="18"/>
+      <c r="H14" s="13"/>
     </row>
     <row r="15" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A15" s="21"/>
-      <c r="B15" s="16">
+      <c r="A15" s="17"/>
+      <c r="B15" s="11">
         <v>3.2</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F15" s="16" t="s">
+      <c r="F15" s="11" t="s">
         <v>51</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H15" s="18"/>
+      <c r="H15" s="13"/>
     </row>
     <row r="16" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A16" s="21"/>
-      <c r="B16" s="16">
+      <c r="A16" s="17"/>
+      <c r="B16" s="11">
         <v>3.3</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="D16" s="16" t="s">
+      <c r="D16" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="E16" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F16" s="16" t="s">
+      <c r="F16" s="11" t="s">
         <v>54</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H16" s="18"/>
+      <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A17" s="21"/>
-      <c r="B17" s="16">
+      <c r="A17" s="17"/>
+      <c r="B17" s="11">
         <v>3.4</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="C17" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="D17" s="16" t="s">
+      <c r="D17" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="E17" s="19" t="s">
+      <c r="E17" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F17" s="16" t="s">
+      <c r="F17" s="11" t="s">
         <v>55</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H17" s="18"/>
+      <c r="H17" s="13"/>
     </row>
     <row r="18" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A18" s="23"/>
-      <c r="B18" s="16">
+      <c r="A18" s="18"/>
+      <c r="B18" s="11">
         <v>3.5</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="C18" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="D18" s="16" t="s">
+      <c r="D18" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="E18" s="17" t="s">
+      <c r="E18" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F18" s="16" t="s">
+      <c r="F18" s="11" t="s">
         <v>60</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H18" s="18"/>
+      <c r="H18" s="13"/>
     </row>
     <row r="19" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="B19" s="16">
+      <c r="B19" s="11">
         <v>4.0999999999999996</v>
       </c>
-      <c r="C19" s="16" t="s">
+      <c r="C19" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="D19" s="16" t="s">
+      <c r="D19" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F19" s="16" t="s">
+      <c r="F19" s="11" t="s">
         <v>64</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H19" s="18"/>
+      <c r="H19" s="13"/>
     </row>
     <row r="20" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A20" s="21"/>
-      <c r="B20" s="16">
+      <c r="A20" s="17"/>
+      <c r="B20" s="11">
         <v>4.2</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="D20" s="16" t="s">
+      <c r="D20" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F20" s="16" t="s">
+      <c r="F20" s="11" t="s">
         <v>65</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H20" s="18"/>
+      <c r="H20" s="13"/>
     </row>
     <row r="21" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A21" s="21"/>
-      <c r="B21" s="16">
+      <c r="A21" s="17"/>
+      <c r="B21" s="11">
         <v>4.3</v>
       </c>
-      <c r="C21" s="16" t="s">
+      <c r="C21" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="D21" s="16" t="s">
+      <c r="D21" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="E21" s="17" t="s">
+      <c r="E21" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F21" s="16" t="s">
+      <c r="F21" s="11" t="s">
         <v>69</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H21" s="18"/>
+      <c r="H21" s="13"/>
     </row>
     <row r="22" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A22" s="21"/>
-      <c r="B22" s="16">
+      <c r="A22" s="17"/>
+      <c r="B22" s="11">
         <v>4.4000000000000004</v>
       </c>
-      <c r="C22" s="16" t="s">
+      <c r="C22" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="D22" s="16" t="s">
+      <c r="D22" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="E22" s="17" t="s">
+      <c r="E22" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F22" s="16" t="s">
+      <c r="F22" s="11" t="s">
         <v>72</v>
       </c>
       <c r="G22" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H22" s="18"/>
+      <c r="H22" s="13"/>
     </row>
     <row r="23" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A23" s="23"/>
-      <c r="B23" s="16">
+      <c r="A23" s="18"/>
+      <c r="B23" s="11">
         <v>4.5</v>
       </c>
-      <c r="C23" s="16" t="s">
+      <c r="C23" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="D23" s="16" t="s">
+      <c r="D23" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="E23" s="17" t="s">
+      <c r="E23" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F23" s="16" t="s">
+      <c r="F23" s="11" t="s">
         <v>75</v>
       </c>
       <c r="G23" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H23" s="18"/>
+      <c r="H23" s="13"/>
     </row>
     <row r="24" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="11">
         <v>5.0999999999999996</v>
       </c>
-      <c r="C24" s="16" t="s">
+      <c r="C24" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="D24" s="16" t="s">
+      <c r="D24" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="E24" s="17" t="s">
+      <c r="E24" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F24" s="16" t="s">
+      <c r="F24" s="11" t="s">
         <v>79</v>
       </c>
       <c r="G24" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H24" s="18"/>
+      <c r="H24" s="13"/>
     </row>
     <row r="25" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A25" s="21"/>
-      <c r="B25" s="16">
+      <c r="A25" s="17"/>
+      <c r="B25" s="11">
         <v>5.2</v>
       </c>
-      <c r="C25" s="16" t="s">
+      <c r="C25" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="D25" s="16" t="s">
+      <c r="D25" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="E25" s="17" t="s">
+      <c r="E25" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F25" s="16" t="s">
+      <c r="F25" s="11" t="s">
         <v>80</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H25" s="18"/>
+      <c r="H25" s="13"/>
     </row>
     <row r="26" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A26" s="21"/>
-      <c r="B26" s="16">
+      <c r="A26" s="17"/>
+      <c r="B26" s="11">
         <v>5.3</v>
       </c>
-      <c r="C26" s="16" t="s">
+      <c r="C26" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="D26" s="16" t="s">
+      <c r="D26" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="E26" s="17" t="s">
+      <c r="E26" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F26" s="16" t="s">
+      <c r="F26" s="11" t="s">
         <v>84</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H26" s="18"/>
+      <c r="H26" s="13"/>
     </row>
     <row r="27" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A27" s="21"/>
-      <c r="B27" s="16">
+      <c r="A27" s="17"/>
+      <c r="B27" s="11">
         <v>5.4</v>
       </c>
-      <c r="C27" s="16" t="s">
+      <c r="C27" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="D27" s="16" t="s">
+      <c r="D27" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="E27" s="17" t="s">
+      <c r="E27" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F27" s="16" t="s">
+      <c r="F27" s="11" t="s">
         <v>87</v>
       </c>
       <c r="G27" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H27" s="18"/>
+      <c r="H27" s="13"/>
     </row>
     <row r="28" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A28" s="21"/>
-      <c r="B28" s="16">
+      <c r="A28" s="17"/>
+      <c r="B28" s="11">
         <v>5.5</v>
       </c>
-      <c r="C28" s="16" t="s">
+      <c r="C28" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="D28" s="16" t="s">
+      <c r="D28" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="E28" s="17" t="s">
+      <c r="E28" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F28" s="16" t="s">
+      <c r="F28" s="11" t="s">
         <v>90</v>
       </c>
       <c r="G28" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H28" s="18"/>
+      <c r="H28" s="13"/>
     </row>
     <row r="29" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A29" s="23"/>
-      <c r="B29" s="16">
+      <c r="A29" s="18"/>
+      <c r="B29" s="11">
         <v>5.6</v>
       </c>
-      <c r="C29" s="16" t="s">
+      <c r="C29" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="D29" s="16" t="s">
+      <c r="D29" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="E29" s="17" t="s">
+      <c r="E29" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F29" s="16" t="s">
+      <c r="F29" s="11" t="s">
         <v>93</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H29" s="18"/>
+      <c r="H29" s="13"/>
     </row>
     <row r="30" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A30" s="22" t="s">
+      <c r="A30" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="11">
         <v>6.1</v>
       </c>
-      <c r="C30" s="16" t="s">
+      <c r="C30" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="D30" s="16" t="s">
+      <c r="D30" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="E30" s="20" t="s">
+      <c r="E30" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="F30" s="16" t="s">
+      <c r="F30" s="11" t="s">
         <v>95</v>
       </c>
       <c r="G30" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="H30" s="13"/>
+    </row>
+    <row r="31" spans="1:8" ht="45" customHeight="1" thickBot="1">
+      <c r="A31" s="17"/>
+      <c r="B31" s="11">
+        <v>6.2</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="D31" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="F31" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="H31" s="13"/>
+    </row>
+    <row r="32" spans="1:8" ht="45" customHeight="1" thickBot="1">
+      <c r="A32" s="17"/>
+      <c r="B32" s="11">
+        <v>6.3</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="D32" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="E32" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="F32" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="H32" s="13"/>
+    </row>
+    <row r="33" spans="1:8" ht="45" customHeight="1" thickBot="1">
+      <c r="A33" s="17"/>
+      <c r="B33" s="11">
+        <v>6.4</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="D33" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="F33" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="G33" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="H30" s="18"/>
-    </row>
-    <row r="31" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A31" s="21"/>
-      <c r="B31" s="16">
-        <v>6.2</v>
-      </c>
-      <c r="C31" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="D31" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="E31" s="20" t="s">
+      <c r="H33" s="13"/>
+    </row>
+    <row r="34" spans="1:8" ht="45" customHeight="1" thickBot="1">
+      <c r="A34" s="17"/>
+      <c r="B34" s="11">
+        <v>6.5</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="D34" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="E34" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="F31" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="G31" s="1" t="s">
+      <c r="F34" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="G34" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="H31" s="18"/>
-    </row>
-    <row r="32" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A32" s="21"/>
-      <c r="B32" s="16">
-        <v>6.3</v>
-      </c>
-      <c r="C32" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="D32" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="E32" s="20" t="s">
+      <c r="H34" s="13"/>
+    </row>
+    <row r="35" spans="1:8" ht="45" customHeight="1" thickBot="1">
+      <c r="A35" s="18"/>
+      <c r="B35" s="11">
+        <v>6.6</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="D35" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="E35" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="F32" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H32" s="18"/>
-    </row>
-    <row r="33" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A33" s="21"/>
-      <c r="B33" s="16">
-        <v>6.4</v>
-      </c>
-      <c r="C33" s="16" t="s">
-        <v>102</v>
-      </c>
-      <c r="D33" s="16" t="s">
-        <v>103</v>
-      </c>
-      <c r="E33" s="20" t="s">
-        <v>97</v>
-      </c>
-      <c r="F33" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="G33" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H33" s="18"/>
-    </row>
-    <row r="34" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A34" s="21"/>
-      <c r="B34" s="16">
-        <v>6.5</v>
-      </c>
-      <c r="C34" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="D34" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="E34" s="20" t="s">
-        <v>97</v>
-      </c>
-      <c r="F34" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H34" s="18"/>
-    </row>
-    <row r="35" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A35" s="23"/>
-      <c r="B35" s="16">
-        <v>6.6</v>
-      </c>
-      <c r="C35" s="16" t="s">
+      <c r="F35" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="D35" s="16" t="s">
-        <v>109</v>
-      </c>
-      <c r="E35" s="20" t="s">
-        <v>97</v>
-      </c>
-      <c r="F35" s="16" t="s">
-        <v>108</v>
-      </c>
       <c r="G35" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H35" s="18"/>
+        <v>210</v>
+      </c>
+      <c r="H35" s="13"/>
     </row>
     <row r="36" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A36" s="22" t="s">
+      <c r="A36" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="B36" s="16">
+      <c r="B36" s="11">
         <v>7.1</v>
       </c>
-      <c r="C36" s="16" t="s">
+      <c r="C36" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="D36" s="16" t="s">
+      <c r="D36" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="E36" s="19" t="s">
+      <c r="E36" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F36" s="16" t="s">
+      <c r="F36" s="11" t="s">
         <v>113</v>
       </c>
       <c r="G36" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H36" s="18"/>
+      <c r="H36" s="13"/>
     </row>
     <row r="37" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A37" s="21"/>
-      <c r="B37" s="16">
+      <c r="A37" s="17"/>
+      <c r="B37" s="11">
         <v>7.2</v>
       </c>
-      <c r="C37" s="16" t="s">
+      <c r="C37" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="D37" s="16" t="s">
+      <c r="D37" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="E37" s="19" t="s">
+      <c r="E37" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F37" s="16" t="s">
+      <c r="F37" s="11" t="s">
         <v>116</v>
       </c>
       <c r="G37" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H37" s="18"/>
+      <c r="H37" s="13"/>
     </row>
     <row r="38" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A38" s="21"/>
-      <c r="B38" s="16">
+      <c r="A38" s="17"/>
+      <c r="B38" s="11">
         <v>7.3</v>
       </c>
-      <c r="C38" s="16" t="s">
+      <c r="C38" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="D38" s="16" t="s">
+      <c r="D38" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="E38" s="19" t="s">
+      <c r="E38" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F38" s="16" t="s">
+      <c r="F38" s="11" t="s">
         <v>119</v>
       </c>
       <c r="G38" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H38" s="18"/>
+      <c r="H38" s="13"/>
     </row>
     <row r="39" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A39" s="21"/>
-      <c r="B39" s="16">
+      <c r="A39" s="17"/>
+      <c r="B39" s="11">
         <v>7.4</v>
       </c>
-      <c r="C39" s="16" t="s">
+      <c r="C39" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="D39" s="16" t="s">
+      <c r="D39" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="E39" s="19" t="s">
+      <c r="E39" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F39" s="16" t="s">
+      <c r="F39" s="11" t="s">
         <v>122</v>
       </c>
       <c r="G39" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H39" s="18"/>
+      <c r="H39" s="13"/>
     </row>
     <row r="40" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A40" s="21"/>
-      <c r="B40" s="16">
+      <c r="A40" s="17"/>
+      <c r="B40" s="11">
         <v>7.5</v>
       </c>
-      <c r="C40" s="16" t="s">
+      <c r="C40" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="D40" s="16" t="s">
+      <c r="D40" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="E40" s="19" t="s">
+      <c r="E40" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F40" s="16" t="s">
+      <c r="F40" s="11" t="s">
         <v>125</v>
       </c>
       <c r="G40" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H40" s="18"/>
+      <c r="H40" s="13"/>
     </row>
     <row r="41" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A41" s="21"/>
-      <c r="B41" s="16">
+      <c r="A41" s="17"/>
+      <c r="B41" s="11">
         <v>7.6</v>
       </c>
-      <c r="C41" s="16" t="s">
+      <c r="C41" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="D41" s="16" t="s">
+      <c r="D41" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="E41" s="19" t="s">
+      <c r="E41" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F41" s="16" t="s">
+      <c r="F41" s="11" t="s">
         <v>128</v>
       </c>
       <c r="G41" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H41" s="18"/>
+      <c r="H41" s="13"/>
     </row>
     <row r="42" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A42" s="23"/>
-      <c r="B42" s="16">
+      <c r="A42" s="18"/>
+      <c r="B42" s="11">
         <v>7.7</v>
       </c>
-      <c r="C42" s="16" t="s">
+      <c r="C42" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="D42" s="16" t="s">
+      <c r="D42" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="E42" s="19" t="s">
+      <c r="E42" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F42" s="16" t="s">
+      <c r="F42" s="11" t="s">
         <v>131</v>
       </c>
       <c r="G42" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H42" s="18"/>
+      <c r="H42" s="13"/>
     </row>
     <row r="43" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A43" s="22" t="s">
+      <c r="A43" s="16" t="s">
         <v>132</v>
       </c>
-      <c r="B43" s="16">
+      <c r="B43" s="11">
         <v>8.1</v>
       </c>
-      <c r="C43" s="16" t="s">
+      <c r="C43" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="D43" s="16" t="s">
+      <c r="D43" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="E43" s="19" t="s">
+      <c r="E43" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F43" s="16" t="s">
+      <c r="F43" s="11" t="s">
         <v>135</v>
       </c>
       <c r="G43" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H43" s="18"/>
+      <c r="H43" s="13"/>
     </row>
     <row r="44" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A44" s="21"/>
-      <c r="B44" s="16">
+      <c r="A44" s="17"/>
+      <c r="B44" s="11">
         <v>8.1999999999999993</v>
       </c>
-      <c r="C44" s="16" t="s">
+      <c r="C44" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="D44" s="16" t="s">
+      <c r="D44" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="E44" s="19" t="s">
+      <c r="E44" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F44" s="16" t="s">
+      <c r="F44" s="11" t="s">
         <v>138</v>
       </c>
       <c r="G44" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H44" s="18"/>
+      <c r="H44" s="13"/>
     </row>
     <row r="45" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A45" s="21"/>
-      <c r="B45" s="16">
+      <c r="A45" s="17"/>
+      <c r="B45" s="11">
         <v>8.3000000000000007</v>
       </c>
-      <c r="C45" s="16" t="s">
+      <c r="C45" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="D45" s="16" t="s">
+      <c r="D45" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="E45" s="19" t="s">
+      <c r="E45" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F45" s="16" t="s">
+      <c r="F45" s="11" t="s">
         <v>141</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H45" s="18"/>
+      <c r="H45" s="13"/>
     </row>
     <row r="46" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A46" s="21"/>
-      <c r="B46" s="16">
+      <c r="A46" s="17"/>
+      <c r="B46" s="11">
         <v>8.4</v>
       </c>
-      <c r="C46" s="16" t="s">
+      <c r="C46" s="11" t="s">
         <v>142</v>
       </c>
-      <c r="D46" s="16" t="s">
+      <c r="D46" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="E46" s="19" t="s">
+      <c r="E46" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F46" s="16" t="s">
+      <c r="F46" s="11" t="s">
         <v>144</v>
       </c>
       <c r="G46" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H46" s="18"/>
+      <c r="H46" s="13"/>
     </row>
     <row r="47" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A47" s="21"/>
-      <c r="B47" s="16">
+      <c r="A47" s="17"/>
+      <c r="B47" s="11">
         <v>8.5</v>
       </c>
-      <c r="C47" s="16" t="s">
+      <c r="C47" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="D47" s="16" t="s">
+      <c r="D47" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="E47" s="19" t="s">
+      <c r="E47" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F47" s="16" t="s">
+      <c r="F47" s="11" t="s">
         <v>147</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H47" s="18"/>
+      <c r="H47" s="13"/>
     </row>
     <row r="48" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A48" s="21"/>
-      <c r="B48" s="16">
+      <c r="A48" s="17"/>
+      <c r="B48" s="11">
         <v>8.6</v>
       </c>
-      <c r="C48" s="16" t="s">
+      <c r="C48" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="D48" s="16" t="s">
+      <c r="D48" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="E48" s="19" t="s">
+      <c r="E48" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F48" s="16" t="s">
+      <c r="F48" s="11" t="s">
         <v>150</v>
       </c>
       <c r="G48" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H48" s="18"/>
+      <c r="H48" s="13"/>
     </row>
     <row r="49" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A49" s="21"/>
-      <c r="B49" s="16">
+      <c r="A49" s="17"/>
+      <c r="B49" s="11">
         <v>8.6999999999999993</v>
       </c>
-      <c r="C49" s="16" t="s">
+      <c r="C49" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="D49" s="16" t="s">
+      <c r="D49" s="11" t="s">
         <v>152</v>
       </c>
-      <c r="E49" s="19" t="s">
+      <c r="E49" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F49" s="16" t="s">
+      <c r="F49" s="11" t="s">
         <v>153</v>
       </c>
       <c r="G49" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H49" s="18"/>
+      <c r="H49" s="13"/>
     </row>
     <row r="50" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A50" s="23"/>
-      <c r="B50" s="16">
+      <c r="A50" s="18"/>
+      <c r="B50" s="11">
         <v>8.8000000000000007</v>
       </c>
-      <c r="C50" s="16" t="s">
+      <c r="C50" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="D50" s="16" t="s">
+      <c r="D50" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="E50" s="19" t="s">
+      <c r="E50" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F50" s="16" t="s">
+      <c r="F50" s="11" t="s">
         <v>156</v>
       </c>
       <c r="G50" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H50" s="18"/>
+      <c r="H50" s="13"/>
     </row>
     <row r="51" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A51" s="22" t="s">
+      <c r="A51" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="B51" s="16">
+      <c r="B51" s="11">
         <v>9.1</v>
       </c>
-      <c r="C51" s="16" t="s">
+      <c r="C51" s="11" t="s">
         <v>158</v>
       </c>
-      <c r="D51" s="16" t="s">
+      <c r="D51" s="11" t="s">
         <v>159</v>
       </c>
-      <c r="E51" s="19" t="s">
+      <c r="E51" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F51" s="16" t="s">
+      <c r="F51" s="11" t="s">
         <v>160</v>
       </c>
       <c r="G51" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H51" s="18"/>
+      <c r="H51" s="13"/>
     </row>
     <row r="52" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A52" s="21"/>
-      <c r="B52" s="16">
+      <c r="A52" s="17"/>
+      <c r="B52" s="11">
         <v>9.1999999999999993</v>
       </c>
-      <c r="C52" s="16" t="s">
+      <c r="C52" s="11" t="s">
         <v>161</v>
       </c>
-      <c r="D52" s="16" t="s">
+      <c r="D52" s="11" t="s">
         <v>162</v>
       </c>
-      <c r="E52" s="19" t="s">
+      <c r="E52" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F52" s="16" t="s">
+      <c r="F52" s="11" t="s">
         <v>163</v>
       </c>
       <c r="G52" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H52" s="18"/>
+      <c r="H52" s="13"/>
     </row>
     <row r="53" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A53" s="21"/>
-      <c r="B53" s="16">
+      <c r="A53" s="17"/>
+      <c r="B53" s="11">
         <v>9.3000000000000007</v>
       </c>
-      <c r="C53" s="16" t="s">
+      <c r="C53" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="D53" s="16" t="s">
+      <c r="D53" s="11" t="s">
         <v>165</v>
       </c>
-      <c r="E53" s="19" t="s">
+      <c r="E53" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F53" s="16" t="s">
+      <c r="F53" s="11" t="s">
         <v>166</v>
       </c>
       <c r="G53" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H53" s="18"/>
+      <c r="H53" s="13"/>
     </row>
     <row r="54" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A54" s="21"/>
-      <c r="B54" s="16">
+      <c r="A54" s="17"/>
+      <c r="B54" s="11">
         <v>9.4</v>
       </c>
-      <c r="C54" s="16" t="s">
+      <c r="C54" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="D54" s="16" t="s">
+      <c r="D54" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="E54" s="19" t="s">
+      <c r="E54" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F54" s="16" t="s">
+      <c r="F54" s="11" t="s">
         <v>169</v>
       </c>
       <c r="G54" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H54" s="18"/>
+      <c r="H54" s="13"/>
     </row>
     <row r="55" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A55" s="21"/>
-      <c r="B55" s="16">
+      <c r="A55" s="17"/>
+      <c r="B55" s="11">
         <v>9.5</v>
       </c>
-      <c r="C55" s="16" t="s">
+      <c r="C55" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="D55" s="16" t="s">
+      <c r="D55" s="11" t="s">
         <v>171</v>
       </c>
-      <c r="E55" s="19" t="s">
+      <c r="E55" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F55" s="16" t="s">
+      <c r="F55" s="11" t="s">
         <v>172</v>
       </c>
       <c r="G55" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H55" s="18"/>
+      <c r="H55" s="13"/>
     </row>
     <row r="56" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A56" s="23"/>
-      <c r="B56" s="16">
+      <c r="A56" s="18"/>
+      <c r="B56" s="11">
         <v>9.6</v>
       </c>
-      <c r="C56" s="16" t="s">
+      <c r="C56" s="11" t="s">
         <v>173</v>
       </c>
-      <c r="D56" s="16" t="s">
+      <c r="D56" s="11" t="s">
         <v>174</v>
       </c>
-      <c r="E56" s="19" t="s">
+      <c r="E56" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F56" s="16" t="s">
+      <c r="F56" s="11" t="s">
         <v>175</v>
       </c>
       <c r="G56" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H56" s="18"/>
+      <c r="H56" s="13"/>
     </row>
     <row r="57" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A57" s="22" t="s">
+      <c r="A57" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="B57" s="16">
+      <c r="B57" s="11">
         <v>10.1</v>
       </c>
-      <c r="C57" s="16" t="s">
+      <c r="C57" s="11" t="s">
         <v>177</v>
       </c>
-      <c r="D57" s="16" t="s">
+      <c r="D57" s="11" t="s">
         <v>178</v>
       </c>
-      <c r="E57" s="19" t="s">
+      <c r="E57" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F57" s="16" t="s">
+      <c r="F57" s="11" t="s">
         <v>177</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H57" s="18"/>
+      <c r="H57" s="13"/>
     </row>
     <row r="58" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A58" s="21"/>
-      <c r="B58" s="16">
+      <c r="A58" s="17"/>
+      <c r="B58" s="11">
         <v>10.199999999999999</v>
       </c>
-      <c r="C58" s="16" t="s">
+      <c r="C58" s="11" t="s">
         <v>179</v>
       </c>
-      <c r="D58" s="16" t="s">
+      <c r="D58" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="E58" s="19" t="s">
+      <c r="E58" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F58" s="16" t="s">
+      <c r="F58" s="11" t="s">
         <v>181</v>
       </c>
       <c r="G58" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H58" s="18"/>
+      <c r="H58" s="13"/>
     </row>
     <row r="59" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A59" s="21"/>
-      <c r="B59" s="16">
+      <c r="A59" s="17"/>
+      <c r="B59" s="11">
         <v>10.3</v>
       </c>
-      <c r="C59" s="16" t="s">
+      <c r="C59" s="11" t="s">
         <v>182</v>
       </c>
-      <c r="D59" s="16" t="s">
+      <c r="D59" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="E59" s="19" t="s">
+      <c r="E59" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F59" s="16" t="s">
+      <c r="F59" s="11" t="s">
         <v>184</v>
       </c>
       <c r="G59" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H59" s="18"/>
+      <c r="H59" s="13"/>
     </row>
     <row r="60" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A60" s="21"/>
-      <c r="B60" s="16">
+      <c r="A60" s="17"/>
+      <c r="B60" s="11">
         <v>10.4</v>
       </c>
-      <c r="C60" s="16" t="s">
+      <c r="C60" s="11" t="s">
         <v>185</v>
       </c>
-      <c r="D60" s="16" t="s">
+      <c r="D60" s="11" t="s">
         <v>186</v>
       </c>
-      <c r="E60" s="19" t="s">
+      <c r="E60" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F60" s="16" t="s">
+      <c r="F60" s="11" t="s">
         <v>187</v>
       </c>
       <c r="G60" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H60" s="18"/>
+      <c r="H60" s="13"/>
     </row>
     <row r="61" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A61" s="23"/>
-      <c r="B61" s="16">
+      <c r="A61" s="18"/>
+      <c r="B61" s="11">
         <v>10.5</v>
       </c>
-      <c r="C61" s="16" t="s">
+      <c r="C61" s="11" t="s">
         <v>188</v>
       </c>
-      <c r="D61" s="16" t="s">
+      <c r="D61" s="11" t="s">
         <v>189</v>
       </c>
-      <c r="E61" s="17" t="s">
+      <c r="E61" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F61" s="16" t="s">
+      <c r="F61" s="11" t="s">
         <v>190</v>
       </c>
       <c r="G61" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H61" s="18"/>
+      <c r="H61" s="13"/>
     </row>
     <row r="62" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A62" s="22" t="s">
+      <c r="A62" s="16" t="s">
         <v>191</v>
       </c>
-      <c r="B62" s="16">
+      <c r="B62" s="11">
         <v>11.1</v>
       </c>
-      <c r="C62" s="16" t="s">
+      <c r="C62" s="11" t="s">
         <v>192</v>
       </c>
-      <c r="D62" s="16" t="s">
+      <c r="D62" s="11" t="s">
         <v>193</v>
       </c>
-      <c r="E62" s="17" t="s">
+      <c r="E62" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F62" s="16" t="s">
+      <c r="F62" s="11" t="s">
         <v>194</v>
       </c>
       <c r="G62" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H62" s="18"/>
+      <c r="H62" s="13"/>
     </row>
     <row r="63" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A63" s="21"/>
-      <c r="B63" s="16">
+      <c r="A63" s="17"/>
+      <c r="B63" s="11">
         <v>11.2</v>
       </c>
-      <c r="C63" s="16" t="s">
+      <c r="C63" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="D63" s="16" t="s">
+      <c r="D63" s="11" t="s">
         <v>196</v>
       </c>
-      <c r="E63" s="17" t="s">
+      <c r="E63" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F63" s="16" t="s">
+      <c r="F63" s="11" t="s">
         <v>197</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H63" s="18"/>
+      <c r="H63" s="13"/>
     </row>
     <row r="64" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A64" s="21"/>
-      <c r="B64" s="16">
+      <c r="A64" s="17"/>
+      <c r="B64" s="11">
         <v>11.3</v>
       </c>
-      <c r="C64" s="16" t="s">
+      <c r="C64" s="11" t="s">
         <v>198</v>
       </c>
-      <c r="D64" s="16" t="s">
+      <c r="D64" s="11" t="s">
         <v>199</v>
       </c>
-      <c r="E64" s="19" t="s">
+      <c r="E64" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F64" s="16" t="s">
+      <c r="F64" s="11" t="s">
         <v>200</v>
       </c>
       <c r="G64" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H64" s="18"/>
+      <c r="H64" s="13"/>
     </row>
     <row r="65" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A65" s="21"/>
-      <c r="B65" s="16">
+      <c r="A65" s="17"/>
+      <c r="B65" s="11">
         <v>11.4</v>
       </c>
-      <c r="C65" s="16" t="s">
+      <c r="C65" s="11" t="s">
         <v>201</v>
       </c>
-      <c r="D65" s="16" t="s">
+      <c r="D65" s="11" t="s">
         <v>202</v>
       </c>
-      <c r="E65" s="19" t="s">
+      <c r="E65" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F65" s="16" t="s">
+      <c r="F65" s="11" t="s">
         <v>203</v>
       </c>
       <c r="G65" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H65" s="18"/>
+      <c r="H65" s="13"/>
     </row>
     <row r="66" spans="1:8" ht="45" customHeight="1" thickBot="1">
-      <c r="A66" s="23"/>
-      <c r="B66" s="16">
+      <c r="A66" s="18"/>
+      <c r="B66" s="11">
         <v>11.5</v>
       </c>
-      <c r="C66" s="16" t="s">
+      <c r="C66" s="11" t="s">
         <v>204</v>
       </c>
-      <c r="D66" s="16" t="s">
+      <c r="D66" s="11" t="s">
         <v>205</v>
       </c>
-      <c r="E66" s="17" t="s">
+      <c r="E66" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F66" s="16" t="s">
+      <c r="F66" s="11" t="s">
         <v>206</v>
       </c>
       <c r="G66" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H66" s="18"/>
+      <c r="H66" s="13"/>
     </row>
     <row r="67" spans="1:8" ht="15.75" customHeight="1">
       <c r="B67" s="2"/>
@@ -6362,39 +6088,39 @@
     <mergeCell ref="A36:A42"/>
   </mergeCells>
   <conditionalFormatting sqref="G2:G66">
-    <cfRule type="cellIs" dxfId="16" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="6" operator="equal">
       <formula>"Selesai"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="5" operator="equal">
       <formula>"Sudah Selesai"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
       <formula>"Sudah Selesai"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G66">
-    <cfRule type="cellIs" dxfId="13" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
       <formula>"Sedang Berjalan"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G66">
-    <cfRule type="cellIs" dxfId="12" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="8" operator="equal">
       <formula>"Terhambat"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G66">
-    <cfRule type="cellIs" dxfId="11" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="9" operator="equal">
       <formula>"Belum Mulai"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G66">
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
       <formula>"Sedang Berjalan"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Terhambat"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Terhambat"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6420,22 +6146,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.75" customHeight="1">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="22" t="s">
         <v>207</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
     </row>
     <row r="3" spans="1:8" ht="30" customHeight="1">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="10"/>
+      <c r="B3" s="20"/>
       <c r="C3" s="3" t="s">
         <v>208</v>
       </c>
@@ -6632,7 +6358,7 @@
       </c>
       <c r="E9" s="4">
         <f>COUNTIF(Roadmap!$G$30:$G$35,"Sedang Berjalan")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" s="4">
         <f>COUNTIF(Roadmap!$G$30:$G$35,"Terhambat")</f>
@@ -6640,7 +6366,7 @@
       </c>
       <c r="G9" s="4">
         <f>COUNTIF(Roadmap!$G$30:$G$35,"Belum Mulai")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H9" s="6">
         <f t="shared" si="0"/>
@@ -6808,10 +6534,10 @@
       </c>
     </row>
     <row r="15" spans="1:8" ht="14.5">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="21" t="s">
         <v>234</v>
       </c>
-      <c r="B15" s="10"/>
+      <c r="B15" s="20"/>
       <c r="C15" s="7">
         <f t="shared" ref="C15:G15" si="1">SUM(C4:C14)</f>
         <v>65</v>
@@ -6822,7 +6548,7 @@
       </c>
       <c r="E15" s="7">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" s="7">
         <f t="shared" si="1"/>
@@ -6830,7 +6556,7 @@
       </c>
       <c r="G15" s="7">
         <f t="shared" si="1"/>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H15" s="8">
         <f t="shared" si="0"/>

</xml_diff>